<commit_message>
Synchronize experiment content across project
</commit_message>
<xml_diff>
--- a/public/downloads/biovolt-labs-literature-backed-mfc-workbook.xlsx
+++ b/public/downloads/biovolt-labs-literature-backed-mfc-workbook.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="Re5075ed99d7d4ccd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protocol Profiles" sheetId="2" r:id="R437a9649129f47bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiment Metadata" sheetId="3" r:id="R5fdda88006254cbc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Measurement Plan" sheetId="4" r:id="R82c2adad3ff24fc9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Measurements" sheetId="5" r:id="R67be85291fa14a51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calculations" sheetId="6" r:id="R55bd4e34829e4c55"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results" sheetId="7" r:id="Rfee9875d06ec4065"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R1e25b0b62f214717"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protocol Profiles" sheetId="2" r:id="R0ce36338ca764426"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiment Metadata" sheetId="3" r:id="R748ffcdaff0b4bf7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Measurement Plan" sheetId="4" r:id="Rff729980fd644687"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Measurements" sheetId="5" r:id="R8ef488acf3fe4863"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calculations" sheetId="6" r:id="R4fe1fffa8dbb425b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results" sheetId="7" r:id="Rb2d1a6b9b25545e6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -590,16 +590,16 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="18" t="str">
-        <x:v>Incomplete prior experiment</x:v>
+        <x:v>Incomplete prior voltage record</x:v>
       </x:c>
       <x:c r="B15" s="18" t="str">
-        <x:v>Do not infer a duration or sampling interval</x:v>
+        <x:v>Retain the recorded 72-hour duration; do not infer a sampling interval</x:v>
       </x:c>
       <x:c r="C15" s="18" t="str">
-        <x:v>Only a single voltage reading was retained</x:v>
+        <x:v>Only a single voltage reading was retained; no continuous time series</x:v>
       </x:c>
       <x:c r="D15" s="18" t="str">
-        <x:v>Blank plan until selected</x:v>
+        <x:v>Duration retained; logging plan blank until selected</x:v>
       </x:c>
       <x:c r="E15" s="2"/>
       <x:c r="F15" s="2"/>
@@ -6925,8 +6925,9 @@
       <x:c r="A5" s="20" t="str">
         <x:v>Selected protocol</x:v>
       </x:c>
-      <x:c r="B5" s="2" t="str">
+      <x:c r="B5" s="2" t="n">
         <x:f>'Experiment Metadata'!B8</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C5" s="2" t="str">
         <x:v>Protocol_ID</x:v>

</xml_diff>